<commit_message>
fix(v1.1): priorizacao de formatacao condicional por status/fiscal e classificacao 'Noturno' quando ha dono
- Ajusta a ordem de precedencia das regras de formatacao condicional na planilha e no template para priorizar status finalizados/em andamento e fiscal atribuido antes das cores de livre/restricao.
- Define Tipo de Servico como 'Noturno' (em vez de 'Noturno Livre') quando o protocolo noturno ja possui fiscal atribuido no fluxo seco, importacao historica e geracao da planilha.
</commit_message>
<xml_diff>
--- a/templates/template_triagem.xlsx
+++ b/templates/template_triagem.xlsx
@@ -78,8 +78,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFC000"/>
-          <bgColor rgb="FFFFC000"/>
+          <fgColor rgb="FF9BBB59"/>
+          <bgColor rgb="FF9BBB59"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD99694"/>
+          <bgColor rgb="FFD99694"/>
         </patternFill>
       </fill>
     </dxf>
@@ -102,6 +110,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFB9CDE5"/>
+          <bgColor rgb="FFB9CDE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FF8064A2"/>
           <bgColor rgb="FF8064A2"/>
         </patternFill>
@@ -110,16 +126,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF9BBB59"/>
-          <bgColor rgb="FF9BBB59"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD99694"/>
-          <bgColor rgb="FFD99694"/>
+          <fgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -128,14 +136,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFF79646"/>
           <bgColor rgb="FFF79646"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB9CDE5"/>
-          <bgColor rgb="FFB9CDE5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -711,49 +711,49 @@
   <autoFilter ref="A2:AF2"/>
   <conditionalFormatting sqref="A3:AF5000">
     <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$B3="Em Andamento"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$B3="Indeferido"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>$B3="Cancelado"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>$B3="Cassado"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>$B3="Deferido"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>$P3="INDEFERIDO"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="2">
+      <formula>$P3="CANCELADO"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="3">
+      <formula>$D3="Noturno entregue"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="4">
+      <formula>$C3&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="5">
+      <formula>$D3="Noturno Livre"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="5">
+      <formula>$E3="Noturno"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="6">
       <formula>$D3="Sem Restrição Livre"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="0">
+    <cfRule type="expression" priority="13" dxfId="6">
       <formula>$E3="Sem Restrição"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="1">
-      <formula>$P3="INDEFERIDO"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
-      <formula>$P3="CANCELADO"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="2">
-      <formula>$D3="Noturno entregue"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="3">
-      <formula>$D3="Noturno Livre"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="3">
-      <formula>$E3="Noturno"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="4">
-      <formula>$B3="Em Andamento"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="9" dxfId="5">
-      <formula>$B3="Indeferido"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="5">
-      <formula>$B3="Cancelado"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="11" dxfId="5">
-      <formula>$B3="Cassado"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="5">
-      <formula>$B3="Deferido"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="13" dxfId="6">
+    <cfRule type="expression" priority="14" dxfId="7">
       <formula>$D3="Com Restrição Livre"</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" dxfId="6">
+    <cfRule type="expression" priority="15" dxfId="7">
       <formula>$E3="Com Restrição"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="15" dxfId="7">
-      <formula>$C3&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>